<commit_message>
Minor improvments for excel_diff
- Rework OS_Process API
- Fix Str API bug
- Add program arguments for excel_diff
</commit_message>
<xml_diff>
--- a/data/bench_disk_base.xlsx
+++ b/data/bench_disk_base.xlsx
@@ -9,17 +9,18 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="930" yWindow="0" windowWidth="37470" windowHeight="18420"/>
+    <workbookView xWindow="1860" yWindow="0" windowWidth="37470" windowHeight="18420" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="bench_disk" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>4KB</t>
   </si>
@@ -73,6 +74,48 @@
   </si>
   <si>
     <t>RND Q32</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Damage</t>
+  </si>
+  <si>
+    <t>Mana</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Level</t>
+  </si>
+  <si>
+    <t>Fire Ball</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>Frost Spear</t>
+  </si>
+  <si>
+    <t>Earthquake</t>
+  </si>
+  <si>
+    <t>Tsunami</t>
   </si>
 </sst>
 </file>
@@ -556,8 +599,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1169,4 +1213,117 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="18.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2">
+        <v>1000</v>
+      </c>
+      <c r="D2">
+        <v>500</v>
+      </c>
+      <c r="E2">
+        <v>10000</v>
+      </c>
+      <c r="F2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3">
+        <v>1500</v>
+      </c>
+      <c r="D3">
+        <v>1000</v>
+      </c>
+      <c r="E3">
+        <v>2500</v>
+      </c>
+      <c r="F3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4">
+        <v>500</v>
+      </c>
+      <c r="D4">
+        <v>10</v>
+      </c>
+      <c r="E4">
+        <v>1000</v>
+      </c>
+      <c r="F4">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5">
+        <v>9999</v>
+      </c>
+      <c r="D5">
+        <v>9999</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>99</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>